<commit_message>
Re-run health insurance recovery with PDF dependencies
</commit_message>
<xml_diff>
--- a/08_Reports - Доклади - Berichte/Accounting_Cash_Flow/enrico_cross_check.xlsx
+++ b/08_Reports - Доклади - Berichte/Accounting_Cash_Flow/enrico_cross_check.xlsx
@@ -937,17 +937,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2022-12</t>
+          <t>2002-01</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t/>
+          <t>2023083</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Gutschrift</t>
+          <t>RECHNUNG</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -957,39 +957,39 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>12.12</t>
+          <t>49.94</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/12-2022 #9120.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/10. Nachweis von Lohnzahlungen - Bankkontoumsätze 2023.pdf</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>REVIEW_ENRICO_DOCUMENT</t>
+          <t>POSSIBLE_MISSING_ENRICO_EVIDENCE</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>2002-01</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2810</t>
+          <t>RG-2024-0</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Rechnung</t>
+          <t>GUTSCHRIFT</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -999,12 +999,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>30.06</t>
+          <t>482.79</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Zahlungsavis Zahariev Juni 2025.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/10. Nachweis von Lohnzahlungen - Bankkontoumsätze 2024.pdf</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1021,17 +1021,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2036-08</t>
+          <t>2022-12</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>02036</t>
+          <t/>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Rechnung</t>
+          <t>Gutschrift</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1041,34 +1041,34 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>675.92</t>
+          <t>12.12</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Martin Zahariev Transporte 2036 08.01.2025 Scannermiete.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/12-2022 #9120.pdf</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t/>
+          <t>REVIEW_ENRICO_DOCUMENT</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2054-07</t>
+          <t>2025-07</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>02054</t>
+          <t>2810</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1083,34 +1083,34 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>637.84</t>
+          <t>30.06</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Martin Zahariev Transporte 2054 07.02.2025 Scannermiete.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/06_Bank_Payments/Zahlungsavis Zahariev Juni 2025.pdf</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t/>
+          <t>POSSIBLE_MISSING_ENRICO_EVIDENCE</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2058-08</t>
+          <t>2036-08</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>02068</t>
+          <t>02036</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1125,12 +1125,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>637.84</t>
+          <t>675.92</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Martin Zahariev Transporte 2058 08.03.2025 Scannermiete.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Martin Zahariev Transporte 2036 08.01.2025 Scannermiete.pdf</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1147,12 +1147,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2054-07</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>02765</t>
+          <t>02054</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2765 Zahariev Hermes Scannermiete.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Martin Zahariev Transporte 2054 07.02.2025 Scannermiete.pdf</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1189,12 +1189,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2058-08</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>02777</t>
+          <t>02068</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1209,34 +1209,34 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>499.80</t>
+          <t>637.84</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2777 Zahariev Hermes Unterstützungstouren.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Martin Zahariev Transporte 2058 08.03.2025 Scannermiete.pdf</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>POSSIBLE_MISSING_ENRICO_EVIDENCE</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2025-04</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>02778</t>
+          <t>02765</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1251,22 +1251,22 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>599.76</t>
+          <t>637.84</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2778 Zahariev Hermes Scannermiete.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2765 Zahariev Hermes Scannermiete.pdf</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>POSSIBLE_MISSING_ENRICO_EVIDENCE</t>
+          <t/>
         </is>
       </c>
     </row>
@@ -1278,7 +1278,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>02782</t>
+          <t>02777</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1293,12 +1293,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>35.70</t>
+          <t>499.80</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2782 Zahariev Hermes Bearbeitungsgebühr.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2777 Zahariev Hermes Unterstützungstouren.pdf</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1315,12 +1315,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>02788</t>
+          <t>02778</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1335,12 +1335,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>523.60</t>
+          <t>599.76</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2788 Zahariev Hermes Scannermiete.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2778 Zahariev Hermes Scannermiete.pdf</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1357,12 +1357,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>02789</t>
+          <t>02782</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1377,12 +1377,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>8282.40</t>
+          <t>35.70</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2789 Zahariev TF Touren.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2782 Zahariev Hermes Bearbeitungsgebühr.pdf</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1404,7 +1404,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>02794</t>
+          <t>02788</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1419,12 +1419,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>71.40</t>
+          <t>523.60</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2794 Zahariev KFZ Miete.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2788 Zahariev Hermes Scannermiete.pdf</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>02799</t>
+          <t>02789</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1461,12 +1461,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>53.55</t>
+          <t>8282.40</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2799 Bearbeitungsgebühr 10.06.2025 Zahariev.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2789 Zahariev TF Touren.pdf</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1483,12 +1483,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>2025-06</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>02810</t>
+          <t>02794</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1503,34 +1503,34 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>9496.20</t>
+          <t>71.40</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2810 Zahariev TF Touren.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2794 Zahariev KFZ Miete.pdf</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t/>
+          <t>POSSIBLE_MISSING_ENRICO_EVIDENCE</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>2025-06</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>02811</t>
+          <t>02799</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1545,22 +1545,22 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>333.20</t>
+          <t>53.55</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2811 Zahariev scannermiete.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2799 Bearbeitungsgebühr 10.06.2025 Zahariev.pdf</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t/>
+          <t>POSSIBLE_MISSING_ENRICO_EVIDENCE</t>
         </is>
       </c>
     </row>
@@ -1572,7 +1572,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>02813</t>
+          <t>02810</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1587,12 +1587,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>47.60</t>
+          <t>9496.20</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2813 zahariev bearbeitungsgebühr.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2810 Zahariev TF Touren.pdf</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>02814</t>
+          <t>02811</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1629,12 +1629,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>166.60</t>
+          <t>333.20</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2814 zahariev bekleidung.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2811 Zahariev scannermiete.pdf</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1651,96 +1651,96 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2023-10</t>
+          <t>2025-07</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>120-2300157425</t>
+          <t>02813</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>GUTSCHRIFT</t>
+          <t>Rechnung</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>26.10.2023</t>
+          <t/>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2034.28</t>
+          <t>47.60</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2300157425.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2813 zahariev bearbeitungsgebühr.pdf</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>POSSIBLE_MISSING_ENRICO_EVIDENCE</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2023-10</t>
+          <t>2025-07</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>120-2300157934</t>
+          <t>02814</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>GUTSCHRIFT</t>
+          <t>Rechnung</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>30.10.2023</t>
+          <t/>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>176843.58</t>
+          <t>166.60</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2300157934.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Rechnung 2814 zahariev bekleidung.pdf</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>POSSIBLE_MISSING_ENRICO_EVIDENCE</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2023-10</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>120-2400000826</t>
+          <t>120-2300157425</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1750,17 +1750,17 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>31.01.2024</t>
+          <t>26.10.2023</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>119991.48</t>
+          <t>2034.28</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400000826.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2300157425.pdf</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1777,12 +1777,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2023-10</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>120-2400000990</t>
+          <t>120-2300157934</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1792,17 +1792,17 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>31.01.2024</t>
+          <t>30.10.2023</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>34171.33</t>
+          <t>176843.58</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400000990.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2300157934.pdf</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1824,7 +1824,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>120-2400001108</t>
+          <t>120-2400000826</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1834,17 +1834,17 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>02.02.2024</t>
+          <t>31.01.2024</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>6242.25</t>
+          <t>119991.48</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400001108-1.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400000826.pdf</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1861,12 +1861,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2024-02</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>120-2400017841</t>
+          <t>120-2400000990</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1876,17 +1876,17 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>21.02.2024</t>
+          <t>31.01.2024</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>634.21</t>
+          <t>34171.33</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400017841.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400000990.pdf</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -1903,12 +1903,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2024-02</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>120-2400018211</t>
+          <t>120-2400001108</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1918,17 +1918,17 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>29.02.2024</t>
+          <t>02.02.2024</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>4.90</t>
+          <t>6242.25</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400018211.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400001108-1.pdf</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -1945,12 +1945,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2024-02</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>120-2400035414</t>
+          <t>120-2400017841</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1960,17 +1960,17 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>26.03.2024</t>
+          <t>21.02.2024</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2543.30</t>
+          <t>634.21</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400035414.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400017841.pdf</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -1987,12 +1987,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2024-01</t>
+          <t>2024-02</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>120-2400035649</t>
+          <t>120-2400018211</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2002,17 +2002,17 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>26.03.2024</t>
+          <t>29.02.2024</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>608.64</t>
+          <t>4.90</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400035649.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400018211.pdf</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2029,84 +2029,84 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2024-07</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>7-2024</t>
+          <t>120-2400035414</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Gutschrift</t>
+          <t>GUTSCHRIFT</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>02.04.2024</t>
+          <t>26.03.2024</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2.06</t>
+          <t>2543.30</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Docutain Dokument.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400035414.pdf</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t/>
+          <t>POSSIBLE_MISSING_ENRICO_EVIDENCE</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2024-01</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>60-2025</t>
+          <t>120-2400035649</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Gutschrift</t>
+          <t>GUTSCHRIFT</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t/>
+          <t>26.03.2024</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>75.91</t>
+          <t>608.64</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift 05.04. 2025 zahariev.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/08_Operating_Costs/Unternehmerabrechnung - VP 120-2400035649.pdf</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t/>
+          <t>POSSIBLE_MISSING_ENRICO_EVIDENCE</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>24-2024</t>
+          <t>7-2024</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2128,39 +2128,39 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t/>
+          <t>02.04.2024</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>179841.96</t>
+          <t>2.06</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 24-2024 Zahariev Martin 31.07.2024.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Docutain Dokument.pdf</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>POSSIBLE_MISSING_ENRICO_EVIDENCE</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2025-04</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>31-2024</t>
+          <t>60-2025</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2175,12 +2175,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>176234.29</t>
+          <t>75.91</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 31-2024 Zahariev Martin 30.09.2024.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift 05.04. 2025 zahariev.pdf</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2197,12 +2197,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2024-10</t>
+          <t>2024-07</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>34-2024</t>
+          <t>24-2024</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2217,34 +2217,34 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>916.00</t>
+          <t>179841.96</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 34-2024 Zahariev Martin 04.10.2024.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 24-2024 Zahariev Martin 31.07.2024.pdf</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t/>
+          <t>POSSIBLE_MISSING_ENRICO_EVIDENCE</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2024-10</t>
+          <t>2024-09</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>38-2024</t>
+          <t>31-2024</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2259,12 +2259,12 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>197442.02</t>
+          <t>176234.29</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 38-2024 Zahariev Martin 31.10.2024.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 31-2024 Zahariev Martin 30.09.2024.pdf</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -2281,12 +2281,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2024-11</t>
+          <t>2024-10</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>42-2024</t>
+          <t>34-2024</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2301,12 +2301,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>232318.76</t>
+          <t>916.00</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 42-2024 Zahariev Martin 30.11.2024.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 34-2024 Zahariev Martin 04.10.2024.pdf</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -2323,12 +2323,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2024-12</t>
+          <t>2024-10</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>44-2024</t>
+          <t>38-2024</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2343,12 +2343,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>188941.38</t>
+          <t>197442.02</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 44-2024 Zahariev Martin 31.12.2024.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 38-2024 Zahariev Martin 31.10.2024.pdf</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2365,12 +2365,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2024-11</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>66-2025</t>
+          <t>42-2024</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2385,12 +2385,12 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>120491.84</t>
+          <t>232318.76</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift 66 Mai 2025 zahariev.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 42-2024 Zahariev Martin 30.11.2024.pdf</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -2407,12 +2407,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2024-12</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>71-2025</t>
+          <t>44-2024</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2427,12 +2427,12 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>50.00</t>
+          <t>188941.38</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift 71 2025 zahariev Sendungsverlust.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift 44-2024 Zahariev Martin 31.12.2024.pdf</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2449,12 +2449,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>61-2025</t>
+          <t>66-2025</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2469,34 +2469,34 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>181792.36</t>
+          <t>120491.84</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift April 2025 zahariev.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift 66 Mai 2025 zahariev.pdf</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>POSSIBLE_MISSING_ENRICO_EVIDENCE</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>2025-06</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>57-2025</t>
+          <t>71-2025</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2511,12 +2511,12 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>202395.66</t>
+          <t>50.00</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift märz 2025 zahariev.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift 71 2025 zahariev Sendungsverlust.pdf</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2533,12 +2533,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2025-04</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>74-2025</t>
+          <t>61-2025</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2553,12 +2553,12 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>55392.95</t>
+          <t>181792.36</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift Zahariev 74 30.06.2025.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift April 2025 zahariev.pdf</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -2575,17 +2575,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2024-12</t>
+          <t>2025-03</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t/>
+          <t>57-2025</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t/>
+          <t>Gutschrift</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2595,39 +2595,39 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t/>
+          <t>202395.66</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Dezember Zahariev 2024.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/gutschrift märz 2025 zahariev.pdf</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>REVIEW_ENRICO_DOCUMENT</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>2025-06</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t/>
+          <t>74-2025</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t/>
+          <t>Gutschrift</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2637,29 +2637,29 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t/>
+          <t>55392.95</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Martin Zahariev Februar 2025.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Gutschrift Zahariev 74 30.06.2025.pdf</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>UNKNOWN</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>REVIEW_ENRICO_DOCUMENT</t>
+          <t>POSSIBLE_MISSING_ENRICO_EVIDENCE</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2025-01</t>
+          <t>2024-12</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2684,7 +2684,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Martin Zahariev Januar 2025.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Dezember Zahariev 2024.pdf</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -2701,7 +2701,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2024-11</t>
+          <t>2025-02</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis November 2024.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Martin Zahariev Februar 2025.pdf</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -2743,7 +2743,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2024-10</t>
+          <t>2025-01</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Oktober 2024.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Martin Zahariev Januar 2025.pdf</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -2785,7 +2785,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2024-09</t>
+          <t>2024-11</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis September 2024.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis November 2024.pdf</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -2827,7 +2827,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>2024-10</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Subunternehmer Sachsenpower GmbH &amp; Co. KG.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Oktober 2024.pdf</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -2869,7 +2869,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2024-09</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2894,7 +2894,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Zahariev April 25 Sachsenpower GmbH &amp; Co. KG.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis September 2024.pdf</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -2911,7 +2911,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2024-07</t>
+          <t>2025-03</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2936,7 +2936,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Zahariev Juli 2024.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Subunternehmer Sachsenpower GmbH &amp; Co. KG.pdf</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -2953,7 +2953,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2025-04</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2978,7 +2978,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Zahariev Juni 25 Sachsenpower GmbH &amp; Co. KG.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Zahariev April 25 Sachsenpower GmbH &amp; Co. KG.pdf</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -2995,7 +2995,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2024-07</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3020,7 +3020,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Zahariev Mai 25 Sachsenpower GmbH &amp; Co. KG.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Zahariev Juli 2024.pdf</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -3037,17 +3037,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2025-01</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>48-2025</t>
+          <t/>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Gutschrift</t>
+          <t/>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -3057,39 +3057,39 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>189578.90</t>
+          <t/>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Gutschrift 48 31.01.2025.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Zahariev Juni 25 Sachsenpower GmbH &amp; Co. KG.pdf</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t/>
+          <t>REVIEW_ENRICO_DOCUMENT</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>2025-05</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>51-2025</t>
+          <t/>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Gutschrift</t>
+          <t/>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -3099,34 +3099,34 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>100.00</t>
+          <t/>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Gutschrift 51 17.02.2025.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Leistungsnachweis Zahariev Mai 25 Sachsenpower GmbH &amp; Co. KG.pdf</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>UNKNOWN</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t/>
+          <t>REVIEW_ENRICO_DOCUMENT</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>2025-01</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>52-2025</t>
+          <t>48-2025</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3141,12 +3141,12 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>170271.25</t>
+          <t>189578.90</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Gutschrift 52 28.02.2025.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Gutschrift 48 31.01.2025.pdf</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -3163,12 +3163,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>2025-02</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>55-2025</t>
+          <t>51-2025</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3183,12 +3183,12 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>95.95</t>
+          <t>100.00</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Gutschrift 55 08.03.2025.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Gutschrift 51 17.02.2025.pdf</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -3205,17 +3205,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2035-08</t>
+          <t>2025-02</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>02035</t>
+          <t>52-2025</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Rechnung</t>
+          <t>Gutschrift</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -3225,12 +3225,12 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>38.00</t>
+          <t>170271.25</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2035 08.01.2025 Hermes Bekleidung.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Gutschrift 52 28.02.2025.pdf</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -3247,17 +3247,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2037-08</t>
+          <t>2025-03</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>02037</t>
+          <t>55-2025</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Rechnung</t>
+          <t>Gutschrift</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -3267,12 +3267,12 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>11648.45</t>
+          <t>95.95</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2037 08.01.2025 Sendungsverluste.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Gutschrift 55 08.03.2025.pdf</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -3289,12 +3289,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2038-08</t>
+          <t>2035-08</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>02038</t>
+          <t>02035</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3309,12 +3309,12 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>181.48</t>
+          <t>38.00</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2038 08.01.2025 Bearbeitungsgebühr.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2035 08.01.2025 Hermes Bekleidung.pdf</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -3331,12 +3331,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2055-07</t>
+          <t>2037-08</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>02055</t>
+          <t>02037</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3351,12 +3351,12 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>7847.85</t>
+          <t>11648.45</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2055 07.02.2025 Sendungsverluste.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2037 08.01.2025 Sendungsverluste.pdf</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -3373,12 +3373,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2056-07</t>
+          <t>2038-08</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>02056</t>
+          <t>02038</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -3393,12 +3393,12 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>163.63</t>
+          <t>181.48</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2056 07.02.2025 Bearbeitungsgebühr.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2038 08.01.2025 Bearbeitungsgebühr.pdf</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -3415,12 +3415,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2057-07</t>
+          <t>2055-07</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>02057</t>
+          <t>02055</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -3435,12 +3435,12 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>94.52</t>
+          <t>7847.85</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2057 07.02.2025 Hermes Bekleidung.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2055 07.02.2025 Sendungsverluste.pdf</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -3457,12 +3457,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2069-08</t>
+          <t>2056-07</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>02069</t>
+          <t>02056</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3477,12 +3477,12 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>2763.67</t>
+          <t>163.63</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2069 08.03.2025 Sendungsverluste.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2056 07.02.2025 Bearbeitungsgebühr.pdf</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -3499,12 +3499,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2070-08</t>
+          <t>2057-07</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>02070</t>
+          <t>02057</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -3519,12 +3519,12 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>98.18</t>
+          <t>94.52</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2070 08.03.2025 Sendungsverluste.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2057 07.02.2025 Hermes Bekleidung.pdf</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -3541,12 +3541,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2024-12</t>
+          <t>2069-08</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>02014</t>
+          <t>02069</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -3561,12 +3561,12 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>10390.09</t>
+          <t>2763.67</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2014 vom 05.12.2024 Sendungsverlust Zahariev.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2069 08.03.2025 Sendungsverluste.pdf</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -3583,12 +3583,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2015-07</t>
+          <t>2070-08</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>02015</t>
+          <t>02070</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -3603,12 +3603,12 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>196.35</t>
+          <t>98.18</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2015 07.12.2024 Martin Zahariev.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Martin Zahariev Transporte 2070 08.03.2025 Sendungsverluste.pdf</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -3630,7 +3630,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>02023</t>
+          <t>02014</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -3645,12 +3645,12 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>50.49</t>
+          <t>10390.09</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2023 vom 07.12.2024  Zahariev HERMES Bekleidung.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2014 vom 05.12.2024 Sendungsverlust Zahariev.pdf</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -3667,12 +3667,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>2015-07</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>02764</t>
+          <t>02015</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -3687,12 +3687,12 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>18.45</t>
+          <t>196.35</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2764 Zahariev Hermes Kleidung.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2015 07.12.2024 Martin Zahariev.pdf</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -3709,12 +3709,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>2024-12</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>02766</t>
+          <t>02023</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -3729,12 +3729,12 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>1545.27</t>
+          <t>50.49</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2766 Zahariev Hermes Sendungsverlust.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2023 vom 07.12.2024  Zahariev HERMES Bekleidung.pdf</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -3756,7 +3756,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>02767</t>
+          <t>02764</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -3771,12 +3771,12 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>50.58</t>
+          <t>18.45</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2767 Zahariev Hermes Bearbeitungsgebuhr.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2764 Zahariev Hermes Kleidung.pdf</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -3793,12 +3793,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>2025-03</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>02781</t>
+          <t>02766</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -3813,34 +3813,34 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>1309.21</t>
+          <t>1545.27</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2781 Zahariev Hermes Sendungsverlust.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2766 Zahariev Hermes Sendungsverlust.pdf</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>POSSIBLE_MISSING_ENRICO_EVIDENCE</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>2025-04</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>02798</t>
+          <t>02767</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -3855,62 +3855,146 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>3042.12</t>
+          <t>50.58</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2798 Zahariev Hermes Sendungsverlust.pdf</t>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2767 Zahariev Hermes Bearbeitungsgebuhr.pdf</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>POSSIBLE_MISSING_ENRICO_EVIDENCE</t>
+          <t/>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>02781</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Rechnung</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>1309.21</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2781 Zahariev Hermes Sendungsverlust.pdf</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>POSSIBLE_MISSING_ENRICO_EVIDENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>02798</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Rechnung</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>3042.12</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2798 Zahariev Hermes Sendungsverlust.pdf</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>POSSIBLE_MISSING_ENRICO_EVIDENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
           <t>2025-07</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
+      <c r="B95" t="inlineStr">
         <is>
           <t>02812</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
+      <c r="C95" t="inlineStr">
         <is>
           <t>Rechnung</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
+      <c r="D95" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
         <is>
           <t>1099.78</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr">
+      <c r="F95" t="inlineStr">
         <is>
           <t>00_INBOX - Входящи - Eingang/Accounting_Organized/09_Enrico_Forwarded/Rechnung 2812 Zahariev Hermes Sendungsverlust.pdf</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr">
+      <c r="G95" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr">
+      <c r="H95" t="inlineStr">
         <is>
           <t>POSSIBLE_MISSING_ENRICO_EVIDENCE</t>
         </is>

</xml_diff>